<commit_message>
feat: refactor pipeline, add date filtering, optimize LLM speed, and remove scheduler daemon
</commit_message>
<xml_diff>
--- a/archives/Issue_2_2026-07-29_職能自動化革命：AI_Agent/stage2_curated_news.xlsx
+++ b/archives/Issue_2_2026-07-29_職能自動化革命：AI_Agent/stage2_curated_news.xlsx
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -786,43 +786,42 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>89 分</t>
+          <t>87 分</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>供應鏈 / 職能自動化 / 供應鏈 / 工作流自動化</t>
+          <t>製造 / 職能自動化 / 製造 / 工作流自動化</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>Walmart如何用數據打造永續零售：AI預測食品浪費，還靠平臺讓供應鏈減碳</t>
+          <t>【2026自動化展】台達如何用 AI-Ready 架構支援跨廠部署與集中管理？</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>2026-07-30 00:00</t>
+          <t>2026-08-24 11:19</t>
         </is>
       </c>
       <c r="F3" s="12" t="inlineStr">
         <is>
-          <t>https://www.ithome.com.tw/news/177760</t>
+          <t>https://techorange.com/2026/08/24/2026automation-delta-ai-ready-linemanager/?utm_source=rss&amp;utm_medium=feed&amp;utm_campaign=techorange_rss</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
         <is>
-          <t>iThome 科技報</t>
+          <t>TechOrange 科技報橘</t>
         </is>
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>對應主題《Walmart如何用數據打造永續零售：A》核心技術落地與實務應用。</t>
+          <t>對應主題《【2026自動化展】台達如何用 AI-R》核心技術落地與實務應用。</t>
         </is>
       </c>
       <c r="I3" s="13" t="inlineStr">
         <is>
-          <t>生成式AI快速發展後，企業開始重新思考AI的價值。對全球最大零售商Walmart而言，AI不只是提升銷售推薦或員工效率的工具，也逐漸成為改善零售流程、降低資源浪費的重要技術。在Walmart最新的FY2026永續報告書，Walmart揭露他們如何利用AI、資料分析、自動化與數位平臺，將永續目標融入日常營運，從食品管理、供應鏈減碳到AI治理，建立以數據驅動的永續零售模式。
-Walmart並非單純以AI解決所有永續問題，而是依照不同場景導入不同數位能力。其中，AI主要用於提升食品管理與營運決策效率，...</t>
+          <t>關稅變化、供應鏈區域化與客戶在地生產需求，促使製造業重新配置全球產能。企業在不同國家設置產線，可縮短供應距離並分散營運風險，據點增加後，設備配置、製程經驗與管理方式也更難維持一致。「製造業目前面臨的重要課題，是如何將既有廠區累積的製造能力、產線經驗與專業知識，快速移轉至其他生產據點。」台達智能製造軟體新事業發展部處長陳鴻輝表示。 台達今年在 2026 台北國際自動化工業大展中，展出一系列針對跨國設廠的部署與管理解決方案。主展位以軟硬體整合方案與應用成果為核心，以 AI-Ready 的智造架構回應...</t>
         </is>
       </c>
     </row>
@@ -832,27 +831,27 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>87 分</t>
+          <t>83 分</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>製造 / 職能自動化 / 製造 / 工作流自動化</t>
+          <t>高階治理 / 職能自動化 / 高階治理 / 工作流自動化</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>【2026自動化展】台達如何用 AI-Ready 架構支援跨廠部署與集中管理？</t>
+          <t>AI Agent 不必全程上雲？Perplexity 聯手 NVIDIA 推 Portable Computer</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>2026-08-24 11:19</t>
+          <t>2026-08-26 18:02</t>
         </is>
       </c>
       <c r="F4" s="12" t="inlineStr">
         <is>
-          <t>https://techorange.com/2026/08/24/2026automation-delta-ai-ready-linemanager/?utm_source=rss&amp;utm_medium=feed&amp;utm_campaign=techorange_rss</t>
+          <t>https://techorange.com/2026/08/26/perplexity-nvidia-portable-computer/?utm_source=rss&amp;utm_medium=feed&amp;utm_campaign=techorange_rss</t>
         </is>
       </c>
       <c r="G4" s="13" t="inlineStr">
@@ -862,12 +861,12 @@
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>對應主題《【2026自動化展】台達如何用 AI-R》核心技術落地與實務應用。</t>
+          <t>對應主題《AI Agent 不必全程上雲？Perp》核心技術落地與實務應用。</t>
         </is>
       </c>
       <c r="I4" s="13" t="inlineStr">
         <is>
-          <t>關稅變化、供應鏈區域化與客戶在地生產需求，促使製造業重新配置全球產能。企業在不同國家設置產線，可縮短供應距離並分散營運風險，據點增加後，設備配置、製程經驗與管理方式也更難維持一致。「製造業目前面臨的重要課題，是如何將既有廠區累積的製造能力、產線經驗與專業知識，快速移轉至其他生產據點。」台達智能製造軟體新事業發展部處長陳鴻輝表示。 台達今年在 2026 台北國際自動化工業大展中，展出一系列針對跨國設廠的部署與管理解決方案。主展位以軟硬體整合方案與應用成果為核心，以 AI-Ready 的智造架構回應...</t>
+          <t>當 AI Agent（AI 代理）開始長時間、自主執行任務後，還適合每一步都靠雲端模型、按 token 付費嗎？和一問一答的聊天機器人不同，Agent 為了完成一項工作，可能持續規劃任務、讀取文件、搜尋資料、呼叫工具，再反覆檢查結果。當工作時間從幾秒拉長到數十分鐘甚至數小時，模型呼叫次數跟著增加，雲端推論成本與資料傳輸問題也會被放大。 Perplexity 現在提出另一種做法，8/25 它與 NVIDIA 推出「Portable Computer」，嘗試把原本依賴雲端執行的 Agent 工作流程...</t>
         </is>
       </c>
     </row>
@@ -877,27 +876,27 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>83 分</t>
+          <t>82 分</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>高階治理 / 職能自動化 / 高階治理 / 工作流自動化</t>
+          <t>財務 / 職能自動化 / 財務 / 工作流自動化</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>AI Agent 不必全程上雲？Perplexity 聯手 NVIDIA 推 Portable Computer</t>
+          <t>【金融 AI 代理安全與防禦】AI Agents 直接經手支付與交易，機構「分階段放權」才是安全底線</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>2026-08-26 18:02</t>
+          <t>2026-08-15 06:29</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>https://techorange.com/2026/08/26/perplexity-nvidia-portable-computer/?utm_source=rss&amp;utm_medium=feed&amp;utm_campaign=techorange_rss</t>
+          <t>https://techorange.com/2026/08/15/securing-ai-agents-in-financial-infrastructure/?utm_source=rss&amp;utm_medium=feed&amp;utm_campaign=techorange_rss</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
@@ -907,12 +906,12 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>對應主題《AI Agent 不必全程上雲？Perp》核心技術落地與實務應用。</t>
+          <t>對應主題《【金融 AI 代理安全與防禦】AI Ag》核心技術落地與實務應用。</t>
         </is>
       </c>
       <c r="I5" s="13" t="inlineStr">
         <is>
-          <t>當 AI Agent（AI 代理）開始長時間、自主執行任務後，還適合每一步都靠雲端模型、按 token 付費嗎？和一問一答的聊天機器人不同，Agent 為了完成一項工作，可能持續規劃任務、讀取文件、搜尋資料、呼叫工具，再反覆檢查結果。當工作時間從幾秒拉長到數十分鐘甚至數小時，模型呼叫次數跟著增加，雲端推論成本與資料傳輸問題也會被放大。 Perplexity 現在提出另一種做法，8/25 它與 NVIDIA 推出「Portable Computer」，嘗試把原本依賴雲端執行的 Agent 工作流程...</t>
+          <t>金融自動化浪潮正以驚人速度席捲。Gartner 預估 2026 年底將有 40% 的企業應用程式，嵌入任務型 AI 代理人（2025 年小於 5%），且已有 79% 企業著手導入。 與僅能生成文字回應的無狀態 Chatbot 不同，AI 代理人結合推理、長期記憶與 API 工具存取，具備自主規劃與執行多步驟任務的能力；這群代理人正深度整合進資金、支付、交易、託管與會計等五大核心領域，從「動口」給資訊轉為直接「動手」運作。 在此高度整合下，代理人任何錯誤決策或惡意操作，都將在數秒內對資產負債表與監...</t>
         </is>
       </c>
     </row>
@@ -922,27 +921,27 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>82 分</t>
+          <t>81 分</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>財務 / 職能自動化 / 財務 / 工作流自動化</t>
+          <t>資安 / 職能自動化 / 資安 / 工作流自動化</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>【金融 AI 代理安全與防禦】AI Agents 直接經手支付與交易，機構「分階段放權」才是安全底線</t>
+          <t>從單點風險到產線韌性，叡揚資訊打造製造業資安閉環：看得見、隔得開、追得完</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>2026-08-15 06:29</t>
+          <t>2026-08-24 17:01</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>https://techorange.com/2026/08/15/securing-ai-agents-in-financial-infrastructure/?utm_source=rss&amp;utm_medium=feed&amp;utm_campaign=techorange_rss</t>
+          <t>https://techorange.com/2026/08/24/gss-bitsight-mendio-codesonar-trackosecops/?utm_source=rss&amp;utm_medium=feed&amp;utm_campaign=techorange_rss</t>
         </is>
       </c>
       <c r="G6" s="13" t="inlineStr">
@@ -952,55 +951,10 @@
       </c>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>對應主題《【金融 AI 代理安全與防禦】AI Ag》核心技術落地與實務應用。</t>
+          <t>對應主題《從單點風險到產線韌性，叡揚資訊打造製造業》核心技術落地與實務應用。</t>
         </is>
       </c>
       <c r="I6" s="13" t="inlineStr">
-        <is>
-          <t>金融自動化浪潮正以驚人速度席捲。Gartner 預估 2026 年底將有 40% 的企業應用程式，嵌入任務型 AI 代理人（2025 年小於 5%），且已有 79% 企業著手導入。 與僅能生成文字回應的無狀態 Chatbot 不同，AI 代理人結合推理、長期記憶與 API 工具存取，具備自主規劃與執行多步驟任務的能力；這群代理人正深度整合進資金、支付、交易、託管與會計等五大核心領域，從「動口」給資訊轉為直接「動手」運作。 在此高度整合下，代理人任何錯誤決策或惡意操作，都將在數秒內對資產負債表與監...</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>81 分</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>資安 / 職能自動化 / 資安 / 工作流自動化</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>從單點風險到產線韌性，叡揚資訊打造製造業資安閉環：看得見、隔得開、追得完</t>
-        </is>
-      </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-24 17:01</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="inlineStr">
-        <is>
-          <t>https://techorange.com/2026/08/24/gss-bitsight-mendio-codesonar-trackosecops/?utm_source=rss&amp;utm_medium=feed&amp;utm_campaign=techorange_rss</t>
-        </is>
-      </c>
-      <c r="G7" s="13" t="inlineStr">
-        <is>
-          <t>TechOrange 科技報橘</t>
-        </is>
-      </c>
-      <c r="H7" s="13" t="inlineStr">
-        <is>
-          <t>對應主題《從單點風險到產線韌性，叡揚資訊打造製造業》核心技術落地與實務應用。</t>
-        </is>
-      </c>
-      <c r="I7" s="13" t="inlineStr">
         <is>
           <t>根據 Gartner 預測，企業若採用持續威脅暴露管理（CTEM），可降低約 67% 的安全漏洞與資安事件，帶動防守戰略從被動回應轉為主動防衛。面對日益嚴峻的資安防禦考驗，叡揚資訊資安直屬事業處技術顧問許農育於日前「半導體供應鏈競爭力論壇」中，以「從一行外部程式碼到一條產線停擺：製造業資安閉環」為題，分析高科技製造業面臨的新型態供應鏈資安威脅，強調企業應建立持續監控與自動化治理能力，從源頭化解隱形風險並確保產線運作穩定。 從攻擊看製造業防禦盲點，建構三層「可視化」架構 現代製造業的資安防護已無法...</t>
         </is>
@@ -1013,7 +967,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>